<commit_message>
updating and adding gitignore finally
</commit_message>
<xml_diff>
--- a/Semester-Planner-101-2026-fall.xlsx
+++ b/Semester-Planner-101-2026-fall.xlsx
@@ -68,7 +68,8 @@
 - rate and gradient</t>
   </si>
   <si>
-    <t xml:space="preserve">Scientific Method</t>
+    <t xml:space="preserve">Scientific Method
+- pendulums</t>
   </si>
   <si>
     <t xml:space="preserve">quiz</t>
@@ -228,7 +229,6 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -250,14 +250,12 @@
       <color rgb="FF000000"/>
       <name val="Open Sans"/>
       <family val="2"/>
-      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FF444444"/>
       <name val="Open Sans"/>
       <family val="2"/>
-      <charset val="1"/>
     </font>
     <font>
       <i val="true"/>
@@ -265,7 +263,6 @@
       <color rgb="FF7F7F7F"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <charset val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -482,6 +479,10 @@
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="166" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -516,10 +517,6 @@
     </xf>
     <xf numFmtId="169" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -552,7 +549,6 @@
     <dxf>
       <font>
         <name val="Calibri"/>
-        <charset val="1"/>
         <family val="2"/>
         <color rgb="FF000000"/>
         <sz val="11"/>
@@ -568,7 +564,6 @@
     <dxf>
       <font>
         <name val="Calibri"/>
-        <charset val="1"/>
         <family val="2"/>
         <color rgb="FF000000"/>
         <sz val="11"/>
@@ -584,7 +579,6 @@
     <dxf>
       <font>
         <name val="Calibri"/>
-        <charset val="1"/>
         <family val="2"/>
         <color rgb="FF000000"/>
         <sz val="11"/>
@@ -600,7 +594,6 @@
     <dxf>
       <font>
         <name val="Calibri"/>
-        <charset val="1"/>
         <family val="2"/>
         <color rgb="FF000000"/>
         <sz val="11"/>
@@ -788,7 +781,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A2:K103"/>
+  <dimension ref="A1:K103"/>
   <sheetFormatPr defaultColWidth="8.8515625" defaultRowHeight="14.4" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10.66"/>
@@ -805,6 +798,7 @@
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1024" min="12" style="1" width="8.84"/>
   </cols>
   <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="s">
         <v>0</v>
@@ -812,7 +806,7 @@
       <c r="C2" s="3"/>
       <c r="D2" s="4"/>
     </row>
-    <row r="3" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="5" t="s">
         <v>1</v>
       </c>
@@ -823,7 +817,7 @@
       <c r="E3" s="7"/>
       <c r="F3" s="8"/>
     </row>
-    <row r="4" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="5" t="s">
         <v>2</v>
       </c>
@@ -843,7 +837,8 @@
         <v>24</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
         <v>4</v>
       </c>
@@ -995,7 +990,7 @@
       <c r="K13" s="18"/>
     </row>
     <row r="14" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="0"/>
+      <c r="A14" s="23"/>
       <c r="B14" s="14" t="n">
         <v>2</v>
       </c>
@@ -1039,7 +1034,7 @@
       <c r="K15" s="18"/>
     </row>
     <row r="16" customFormat="false" ht="15.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="23" t="n">
+      <c r="A16" s="24" t="n">
         <f aca="false">DATE(D3,D4+1,1)</f>
         <v>46266</v>
       </c>
@@ -1060,7 +1055,7 @@
       <c r="J16" s="14"/>
       <c r="K16" s="18"/>
     </row>
-    <row r="17" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="14"/>
       <c r="C17" s="20"/>
       <c r="D17" s="21"/>
@@ -1097,7 +1092,7 @@
       <c r="J18" s="14"/>
       <c r="K18" s="18"/>
     </row>
-    <row r="19" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="14"/>
       <c r="C19" s="20"/>
       <c r="D19" s="21"/>
@@ -1121,7 +1116,7 @@
         <f aca="false">IF(D19="",D18+IF(OR(WEEKDAY(D18)=2,WEEKDAY(D18)=4),2,3),"")</f>
         <v>46272</v>
       </c>
-      <c r="E20" s="24" t="s">
+      <c r="E20" s="25" t="s">
         <v>18</v>
       </c>
       <c r="F20" s="16" t="s">
@@ -1142,11 +1137,11 @@
         <v>20</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="14"/>
       <c r="C21" s="14"/>
       <c r="D21" s="15"/>
-      <c r="E21" s="24"/>
+      <c r="E21" s="25"/>
       <c r="F21" s="16"/>
       <c r="G21" s="16"/>
       <c r="H21" s="15"/>
@@ -1154,7 +1149,7 @@
       <c r="J21" s="14"/>
       <c r="K21" s="18"/>
     </row>
-    <row r="22" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="14"/>
       <c r="C22" s="20" t="n">
         <f aca="false">C20+1</f>
@@ -1172,7 +1167,7 @@
       <c r="J22" s="14"/>
       <c r="K22" s="18"/>
     </row>
-    <row r="23" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="14"/>
       <c r="C23" s="20"/>
       <c r="D23" s="21"/>
@@ -1209,7 +1204,7 @@
       <c r="J24" s="14"/>
       <c r="K24" s="18"/>
     </row>
-    <row r="25" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="14"/>
       <c r="C25" s="20"/>
       <c r="D25" s="21"/>
@@ -1245,14 +1240,14 @@
       <c r="I26" s="14" t="n">
         <v>7</v>
       </c>
-      <c r="J26" s="25" t="n">
+      <c r="J26" s="26" t="n">
         <v>4</v>
       </c>
-      <c r="K26" s="26" t="s">
+      <c r="K26" s="27" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="14"/>
       <c r="C27" s="14"/>
       <c r="D27" s="15"/>
@@ -1262,9 +1257,9 @@
       <c r="H27" s="15"/>
       <c r="I27" s="14"/>
       <c r="J27" s="14"/>
-      <c r="K27" s="26"/>
-    </row>
-    <row r="28" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="K27" s="27"/>
+    </row>
+    <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="14"/>
       <c r="C28" s="20" t="n">
         <f aca="false">C26+1</f>
@@ -1280,24 +1275,24 @@
       <c r="H28" s="15"/>
       <c r="I28" s="14"/>
       <c r="J28" s="14"/>
-      <c r="K28" s="26"/>
-    </row>
-    <row r="29" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="K28" s="27"/>
+    </row>
+    <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="14"/>
       <c r="C29" s="20"/>
       <c r="D29" s="21"/>
       <c r="E29" s="22"/>
       <c r="F29" s="22"/>
-      <c r="G29" s="27"/>
-      <c r="H29" s="28" t="n">
+      <c r="G29" s="28"/>
+      <c r="H29" s="29" t="n">
         <f aca="false">H26+IF(WEEKDAY(H26)=3,2,5)</f>
         <v>46282</v>
       </c>
-      <c r="I29" s="29" t="n">
+      <c r="I29" s="30" t="n">
         <v>8</v>
       </c>
-      <c r="J29" s="25"/>
-      <c r="K29" s="26"/>
+      <c r="J29" s="26"/>
+      <c r="K29" s="27"/>
     </row>
     <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B30" s="14"/>
@@ -1309,27 +1304,27 @@
         <f aca="false">IF(D29="",D28+IF(OR(WEEKDAY(D28)=2,WEEKDAY(D28)=4),2,3),"")</f>
         <v>46283</v>
       </c>
-      <c r="E30" s="27" t="s">
+      <c r="E30" s="28" t="s">
         <v>15</v>
       </c>
       <c r="F30" s="17"/>
-      <c r="G30" s="27"/>
-      <c r="H30" s="28"/>
-      <c r="I30" s="29"/>
-      <c r="J30" s="25"/>
-      <c r="K30" s="26"/>
-    </row>
-    <row r="31" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G30" s="28"/>
+      <c r="H30" s="29"/>
+      <c r="I30" s="30"/>
+      <c r="J30" s="26"/>
+      <c r="K30" s="27"/>
+    </row>
+    <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="14"/>
       <c r="C31" s="20"/>
       <c r="D31" s="21"/>
-      <c r="E31" s="27"/>
+      <c r="E31" s="28"/>
       <c r="F31" s="17"/>
-      <c r="G31" s="27"/>
-      <c r="H31" s="28"/>
-      <c r="I31" s="29"/>
-      <c r="J31" s="25"/>
-      <c r="K31" s="26"/>
+      <c r="G31" s="28"/>
+      <c r="H31" s="29"/>
+      <c r="I31" s="30"/>
+      <c r="J31" s="26"/>
+      <c r="K31" s="27"/>
     </row>
     <row r="32" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B32" s="14" t="n">
@@ -1344,7 +1339,7 @@
         <v>46286</v>
       </c>
       <c r="E32" s="16"/>
-      <c r="F32" s="26" t="s">
+      <c r="F32" s="27" t="s">
         <v>23</v>
       </c>
       <c r="G32" s="16"/>
@@ -1355,14 +1350,14 @@
       <c r="I32" s="14" t="n">
         <v>9</v>
       </c>
-      <c r="J32" s="25" t="n">
+      <c r="J32" s="26" t="n">
         <v>5</v>
       </c>
-      <c r="K32" s="26" t="s">
+      <c r="K32" s="27" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="14"/>
       <c r="C33" s="14"/>
       <c r="D33" s="15"/>
@@ -1372,9 +1367,9 @@
       <c r="H33" s="15"/>
       <c r="I33" s="14"/>
       <c r="J33" s="14"/>
-      <c r="K33" s="26"/>
-    </row>
-    <row r="34" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="K33" s="27"/>
+    </row>
+    <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="14"/>
       <c r="C34" s="20" t="n">
         <f aca="false">C32+1</f>
@@ -1385,29 +1380,29 @@
         <v>46288</v>
       </c>
       <c r="E34" s="22"/>
-      <c r="F34" s="26"/>
+      <c r="F34" s="27"/>
       <c r="G34" s="16"/>
       <c r="H34" s="15"/>
       <c r="I34" s="14"/>
       <c r="J34" s="14"/>
-      <c r="K34" s="26"/>
-    </row>
-    <row r="35" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="K34" s="27"/>
+    </row>
+    <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="14"/>
       <c r="C35" s="20"/>
       <c r="D35" s="21"/>
       <c r="E35" s="22"/>
       <c r="F35" s="22"/>
-      <c r="G35" s="27"/>
-      <c r="H35" s="28" t="n">
+      <c r="G35" s="28"/>
+      <c r="H35" s="29" t="n">
         <f aca="false">H32+IF(WEEKDAY(H32)=3,2,5)</f>
         <v>46289</v>
       </c>
-      <c r="I35" s="29" t="n">
+      <c r="I35" s="30" t="n">
         <v>10</v>
       </c>
-      <c r="J35" s="25"/>
-      <c r="K35" s="26"/>
+      <c r="J35" s="26"/>
+      <c r="K35" s="27"/>
     </row>
     <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B36" s="14"/>
@@ -1419,27 +1414,27 @@
         <f aca="false">IF(D35="",D34+IF(OR(WEEKDAY(D34)=2,WEEKDAY(D34)=4),2,3),"")</f>
         <v>46290</v>
       </c>
-      <c r="E36" s="27" t="s">
+      <c r="E36" s="28" t="s">
         <v>15</v>
       </c>
-      <c r="F36" s="26"/>
-      <c r="G36" s="27"/>
-      <c r="H36" s="28"/>
-      <c r="I36" s="29"/>
-      <c r="J36" s="25"/>
-      <c r="K36" s="26"/>
-    </row>
-    <row r="37" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F36" s="27"/>
+      <c r="G36" s="28"/>
+      <c r="H36" s="29"/>
+      <c r="I36" s="30"/>
+      <c r="J36" s="26"/>
+      <c r="K36" s="27"/>
+    </row>
+    <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="14"/>
       <c r="C37" s="20"/>
       <c r="D37" s="21"/>
-      <c r="E37" s="27"/>
-      <c r="F37" s="26"/>
-      <c r="G37" s="27"/>
-      <c r="H37" s="28"/>
-      <c r="I37" s="29"/>
-      <c r="J37" s="25"/>
-      <c r="K37" s="26"/>
+      <c r="E37" s="28"/>
+      <c r="F37" s="27"/>
+      <c r="G37" s="28"/>
+      <c r="H37" s="29"/>
+      <c r="I37" s="30"/>
+      <c r="J37" s="26"/>
+      <c r="K37" s="27"/>
     </row>
     <row r="38" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="14" t="n">
@@ -1454,7 +1449,7 @@
         <v>46293</v>
       </c>
       <c r="E38" s="16"/>
-      <c r="F38" s="26" t="s">
+      <c r="F38" s="27" t="s">
         <v>25</v>
       </c>
       <c r="G38" s="16"/>
@@ -1465,27 +1460,27 @@
       <c r="I38" s="14" t="n">
         <v>11</v>
       </c>
-      <c r="J38" s="25" t="n">
+      <c r="J38" s="26" t="n">
         <v>6</v>
       </c>
-      <c r="K38" s="26" t="s">
+      <c r="K38" s="27" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="0"/>
+    <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="23"/>
       <c r="B39" s="14"/>
       <c r="C39" s="14"/>
       <c r="D39" s="15"/>
       <c r="E39" s="16"/>
-      <c r="F39" s="26"/>
+      <c r="F39" s="27"/>
       <c r="G39" s="16"/>
       <c r="H39" s="15"/>
       <c r="I39" s="14"/>
       <c r="J39" s="14"/>
-      <c r="K39" s="26"/>
-    </row>
-    <row r="40" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="K39" s="27"/>
+    </row>
+    <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B40" s="14"/>
       <c r="C40" s="20" t="n">
         <f aca="false">C38+1</f>
@@ -1496,34 +1491,34 @@
         <v>46295</v>
       </c>
       <c r="E40" s="22"/>
-      <c r="F40" s="26"/>
+      <c r="F40" s="27"/>
       <c r="G40" s="16"/>
       <c r="H40" s="15"/>
       <c r="I40" s="14"/>
       <c r="J40" s="14"/>
-      <c r="K40" s="26"/>
+      <c r="K40" s="27"/>
     </row>
     <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B41" s="14"/>
       <c r="C41" s="20"/>
       <c r="D41" s="21"/>
       <c r="E41" s="22"/>
-      <c r="F41" s="26"/>
-      <c r="G41" s="27" t="s">
+      <c r="F41" s="27"/>
+      <c r="G41" s="28" t="s">
         <v>27</v>
       </c>
-      <c r="H41" s="28" t="n">
+      <c r="H41" s="29" t="n">
         <f aca="false">H38+IF(WEEKDAY(H38)=3,2,5)</f>
         <v>46296</v>
       </c>
-      <c r="I41" s="29" t="n">
+      <c r="I41" s="30" t="n">
         <v>12</v>
       </c>
-      <c r="J41" s="25"/>
-      <c r="K41" s="26"/>
+      <c r="J41" s="26"/>
+      <c r="K41" s="27"/>
     </row>
     <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="23" t="n">
+      <c r="A42" s="24" t="n">
         <f aca="false">DATE(D3,D4+2,1)</f>
         <v>46296</v>
       </c>
@@ -1536,27 +1531,27 @@
         <f aca="false">IF(D41="",D40+IF(OR(WEEKDAY(D40)=2,WEEKDAY(D40)=4),2,3),"")</f>
         <v>46297</v>
       </c>
-      <c r="E42" s="27" t="s">
+      <c r="E42" s="28" t="s">
         <v>27</v>
       </c>
-      <c r="F42" s="26"/>
-      <c r="G42" s="27"/>
-      <c r="H42" s="28"/>
-      <c r="I42" s="29"/>
-      <c r="J42" s="25"/>
-      <c r="K42" s="26"/>
-    </row>
-    <row r="43" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F42" s="27"/>
+      <c r="G42" s="28"/>
+      <c r="H42" s="29"/>
+      <c r="I42" s="30"/>
+      <c r="J42" s="26"/>
+      <c r="K42" s="27"/>
+    </row>
+    <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B43" s="14"/>
       <c r="C43" s="20"/>
       <c r="D43" s="21"/>
-      <c r="E43" s="27"/>
-      <c r="F43" s="26"/>
-      <c r="G43" s="27"/>
-      <c r="H43" s="28"/>
-      <c r="I43" s="29"/>
-      <c r="J43" s="25"/>
-      <c r="K43" s="26"/>
+      <c r="E43" s="28"/>
+      <c r="F43" s="27"/>
+      <c r="G43" s="28"/>
+      <c r="H43" s="29"/>
+      <c r="I43" s="30"/>
+      <c r="J43" s="26"/>
+      <c r="K43" s="27"/>
     </row>
     <row r="44" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B44" s="14" t="n">
@@ -1582,14 +1577,14 @@
       <c r="I44" s="14" t="n">
         <v>13</v>
       </c>
-      <c r="J44" s="25" t="n">
+      <c r="J44" s="26" t="n">
         <v>7</v>
       </c>
-      <c r="K44" s="26" t="s">
+      <c r="K44" s="27" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="45" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B45" s="14"/>
       <c r="C45" s="14"/>
       <c r="D45" s="15"/>
@@ -1599,9 +1594,9 @@
       <c r="H45" s="15"/>
       <c r="I45" s="14"/>
       <c r="J45" s="14"/>
-      <c r="K45" s="26"/>
-    </row>
-    <row r="46" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="K45" s="27"/>
+    </row>
+    <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B46" s="14"/>
       <c r="C46" s="20" t="n">
         <f aca="false">C44+1</f>
@@ -1617,24 +1612,24 @@
       <c r="H46" s="15"/>
       <c r="I46" s="14"/>
       <c r="J46" s="14"/>
-      <c r="K46" s="26"/>
-    </row>
-    <row r="47" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="K46" s="27"/>
+    </row>
+    <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B47" s="14"/>
       <c r="C47" s="20"/>
       <c r="D47" s="21"/>
       <c r="E47" s="22"/>
       <c r="F47" s="22"/>
-      <c r="G47" s="27"/>
-      <c r="H47" s="28" t="n">
+      <c r="G47" s="28"/>
+      <c r="H47" s="29" t="n">
         <f aca="false">H44+IF(WEEKDAY(H44)=3,2,5)</f>
         <v>46303</v>
       </c>
-      <c r="I47" s="29" t="n">
+      <c r="I47" s="30" t="n">
         <v>14</v>
       </c>
-      <c r="J47" s="25"/>
-      <c r="K47" s="26"/>
+      <c r="J47" s="26"/>
+      <c r="K47" s="27"/>
     </row>
     <row r="48" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B48" s="14"/>
@@ -1646,27 +1641,27 @@
         <f aca="false">IF(D47="",D46+IF(OR(WEEKDAY(D46)=2,WEEKDAY(D46)=4),2,3),"")</f>
         <v>46304</v>
       </c>
-      <c r="E48" s="27" t="s">
+      <c r="E48" s="28" t="s">
         <v>30</v>
       </c>
       <c r="F48" s="17"/>
-      <c r="G48" s="27"/>
-      <c r="H48" s="28"/>
-      <c r="I48" s="29"/>
-      <c r="J48" s="25"/>
-      <c r="K48" s="26"/>
-    </row>
-    <row r="49" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G48" s="28"/>
+      <c r="H48" s="29"/>
+      <c r="I48" s="30"/>
+      <c r="J48" s="26"/>
+      <c r="K48" s="27"/>
+    </row>
+    <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B49" s="14"/>
       <c r="C49" s="20"/>
       <c r="D49" s="21"/>
-      <c r="E49" s="27"/>
+      <c r="E49" s="28"/>
       <c r="F49" s="17"/>
-      <c r="G49" s="27"/>
-      <c r="H49" s="28"/>
-      <c r="I49" s="29"/>
-      <c r="J49" s="25"/>
-      <c r="K49" s="26"/>
+      <c r="G49" s="28"/>
+      <c r="H49" s="29"/>
+      <c r="I49" s="30"/>
+      <c r="J49" s="26"/>
+      <c r="K49" s="27"/>
     </row>
     <row r="50" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B50" s="14" t="n">
@@ -1677,13 +1672,13 @@
         <f aca="false">IF(D49="",D48+IF(OR(WEEKDAY(D48)=2,WEEKDAY(D48)=4),2,3),"")</f>
         <v>46307</v>
       </c>
-      <c r="E50" s="24" t="s">
+      <c r="E50" s="25" t="s">
         <v>31</v>
       </c>
       <c r="F50" s="16" t="s">
         <v>32</v>
       </c>
-      <c r="G50" s="24" t="s">
+      <c r="G50" s="25" t="s">
         <v>31</v>
       </c>
       <c r="H50" s="15" t="n">
@@ -1694,23 +1689,23 @@
       <c r="J50" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="K50" s="30" t="s">
+      <c r="K50" s="31" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="51" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B51" s="14"/>
       <c r="C51" s="14"/>
       <c r="D51" s="15"/>
-      <c r="E51" s="24"/>
+      <c r="E51" s="25"/>
       <c r="F51" s="16"/>
-      <c r="G51" s="24"/>
+      <c r="G51" s="25"/>
       <c r="H51" s="15"/>
       <c r="I51" s="14"/>
       <c r="J51" s="14"/>
-      <c r="K51" s="30"/>
-    </row>
-    <row r="52" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="K51" s="31"/>
+    </row>
+    <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B52" s="14"/>
       <c r="C52" s="20" t="n">
         <v>22</v>
@@ -1721,13 +1716,13 @@
       </c>
       <c r="E52" s="22"/>
       <c r="F52" s="16"/>
-      <c r="G52" s="24"/>
+      <c r="G52" s="25"/>
       <c r="H52" s="15"/>
       <c r="I52" s="14"/>
       <c r="J52" s="14"/>
-      <c r="K52" s="30"/>
-    </row>
-    <row r="53" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="K52" s="31"/>
+    </row>
+    <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B53" s="14"/>
       <c r="C53" s="20"/>
       <c r="D53" s="21"/>
@@ -1738,12 +1733,12 @@
         <f aca="false">H50+IF(WEEKDAY(H50)=3,2,5)</f>
         <v>46310</v>
       </c>
-      <c r="I53" s="29" t="n">
+      <c r="I53" s="30" t="n">
         <f aca="false">I47+1</f>
         <v>15</v>
       </c>
       <c r="J53" s="14"/>
-      <c r="K53" s="30"/>
+      <c r="K53" s="31"/>
     </row>
     <row r="54" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B54" s="14"/>
@@ -1761,11 +1756,11 @@
       <c r="F54" s="16"/>
       <c r="G54" s="22"/>
       <c r="H54" s="21"/>
-      <c r="I54" s="29"/>
+      <c r="I54" s="30"/>
       <c r="J54" s="14"/>
-      <c r="K54" s="30"/>
-    </row>
-    <row r="55" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="K54" s="31"/>
+    </row>
+    <row r="55" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B55" s="14"/>
       <c r="C55" s="20"/>
       <c r="D55" s="21"/>
@@ -1773,12 +1768,12 @@
       <c r="F55" s="16"/>
       <c r="G55" s="22"/>
       <c r="H55" s="21"/>
-      <c r="I55" s="29"/>
+      <c r="I55" s="30"/>
       <c r="J55" s="14"/>
-      <c r="K55" s="30"/>
+      <c r="K55" s="31"/>
     </row>
     <row r="56" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B56" s="25" t="n">
+      <c r="B56" s="26" t="n">
         <v>9</v>
       </c>
       <c r="C56" s="14" t="n">
@@ -1802,15 +1797,15 @@
         <f aca="false">I53+1</f>
         <v>16</v>
       </c>
-      <c r="J56" s="25" t="n">
+      <c r="J56" s="26" t="n">
         <v>9</v>
       </c>
-      <c r="K56" s="26" t="s">
+      <c r="K56" s="27" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="57" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B57" s="25"/>
+    <row r="57" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B57" s="26"/>
       <c r="C57" s="14"/>
       <c r="D57" s="15"/>
       <c r="E57" s="16"/>
@@ -1819,10 +1814,10 @@
       <c r="H57" s="15"/>
       <c r="I57" s="14"/>
       <c r="J57" s="14"/>
-      <c r="K57" s="26"/>
-    </row>
-    <row r="58" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B58" s="25"/>
+      <c r="K57" s="27"/>
+    </row>
+    <row r="58" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B58" s="26"/>
       <c r="C58" s="20" t="n">
         <f aca="false">C56+1</f>
         <v>25</v>
@@ -1837,60 +1832,60 @@
       <c r="H58" s="15"/>
       <c r="I58" s="14"/>
       <c r="J58" s="14"/>
-      <c r="K58" s="26"/>
-    </row>
-    <row r="59" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B59" s="25"/>
+      <c r="K58" s="27"/>
+    </row>
+    <row r="59" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B59" s="26"/>
       <c r="C59" s="20"/>
       <c r="D59" s="21"/>
       <c r="E59" s="22"/>
       <c r="F59" s="22"/>
-      <c r="G59" s="27"/>
-      <c r="H59" s="28" t="n">
+      <c r="G59" s="28"/>
+      <c r="H59" s="29" t="n">
         <f aca="false">H56+IF(WEEKDAY(H56)=3,2,5)</f>
         <v>46317</v>
       </c>
-      <c r="I59" s="29" t="n">
+      <c r="I59" s="30" t="n">
         <f aca="false">I56+1</f>
         <v>17</v>
       </c>
-      <c r="J59" s="25"/>
-      <c r="K59" s="26"/>
+      <c r="J59" s="26"/>
+      <c r="K59" s="27"/>
     </row>
     <row r="60" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B60" s="25"/>
-      <c r="C60" s="31" t="n">
+      <c r="B60" s="26"/>
+      <c r="C60" s="32" t="n">
         <f aca="false">C58+1</f>
         <v>26</v>
       </c>
-      <c r="D60" s="28" t="n">
+      <c r="D60" s="29" t="n">
         <f aca="false">IF(D59="",D58+IF(OR(WEEKDAY(D58)=2,WEEKDAY(D58)=4),2,3),"")</f>
         <v>46318</v>
       </c>
-      <c r="E60" s="27" t="s">
+      <c r="E60" s="28" t="s">
         <v>15</v>
       </c>
       <c r="F60" s="17"/>
-      <c r="G60" s="27"/>
-      <c r="H60" s="28"/>
-      <c r="I60" s="29"/>
-      <c r="J60" s="25"/>
-      <c r="K60" s="26"/>
-    </row>
-    <row r="61" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B61" s="25"/>
-      <c r="C61" s="31"/>
-      <c r="D61" s="28"/>
-      <c r="E61" s="27"/>
+      <c r="G60" s="28"/>
+      <c r="H60" s="29"/>
+      <c r="I60" s="30"/>
+      <c r="J60" s="26"/>
+      <c r="K60" s="27"/>
+    </row>
+    <row r="61" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B61" s="26"/>
+      <c r="C61" s="32"/>
+      <c r="D61" s="29"/>
+      <c r="E61" s="28"/>
       <c r="F61" s="17"/>
-      <c r="G61" s="27"/>
-      <c r="H61" s="28"/>
-      <c r="I61" s="29"/>
-      <c r="J61" s="25"/>
-      <c r="K61" s="26"/>
+      <c r="G61" s="28"/>
+      <c r="H61" s="29"/>
+      <c r="I61" s="30"/>
+      <c r="J61" s="26"/>
+      <c r="K61" s="27"/>
     </row>
     <row r="62" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B62" s="25" t="n">
+      <c r="B62" s="26" t="n">
         <v>10</v>
       </c>
       <c r="C62" s="14" t="n">
@@ -1914,15 +1909,15 @@
         <f aca="false">I59+1</f>
         <v>18</v>
       </c>
-      <c r="J62" s="25" t="n">
+      <c r="J62" s="26" t="n">
         <v>10</v>
       </c>
-      <c r="K62" s="26" t="s">
+      <c r="K62" s="27" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="63" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B63" s="25"/>
+    <row r="63" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B63" s="26"/>
       <c r="C63" s="14"/>
       <c r="D63" s="15"/>
       <c r="E63" s="16"/>
@@ -1931,10 +1926,10 @@
       <c r="H63" s="15"/>
       <c r="I63" s="14"/>
       <c r="J63" s="14"/>
-      <c r="K63" s="26"/>
-    </row>
-    <row r="64" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B64" s="25"/>
+      <c r="K63" s="27"/>
+    </row>
+    <row r="64" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B64" s="26"/>
       <c r="C64" s="20" t="n">
         <f aca="false">C62+1</f>
         <v>28</v>
@@ -1949,65 +1944,65 @@
       <c r="H64" s="15"/>
       <c r="I64" s="14"/>
       <c r="J64" s="14"/>
-      <c r="K64" s="26"/>
-    </row>
-    <row r="65" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B65" s="25"/>
+      <c r="K64" s="27"/>
+    </row>
+    <row r="65" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B65" s="26"/>
       <c r="C65" s="20"/>
       <c r="D65" s="21"/>
       <c r="E65" s="22"/>
       <c r="F65" s="22"/>
-      <c r="G65" s="27"/>
-      <c r="H65" s="28" t="n">
+      <c r="G65" s="28"/>
+      <c r="H65" s="29" t="n">
         <f aca="false">H62+IF(WEEKDAY(H62)=3,2,5)</f>
         <v>46324</v>
       </c>
-      <c r="I65" s="29" t="n">
+      <c r="I65" s="30" t="n">
         <f aca="false">I62+1</f>
         <v>19</v>
       </c>
-      <c r="J65" s="25"/>
-      <c r="K65" s="26"/>
+      <c r="J65" s="26"/>
+      <c r="K65" s="27"/>
     </row>
     <row r="66" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A66" s="32"/>
-      <c r="B66" s="25"/>
-      <c r="C66" s="31" t="n">
+      <c r="A66" s="23"/>
+      <c r="B66" s="26"/>
+      <c r="C66" s="32" t="n">
         <f aca="false">C64+1</f>
         <v>29</v>
       </c>
-      <c r="D66" s="28" t="n">
+      <c r="D66" s="29" t="n">
         <f aca="false">IF(D65="",D64+IF(OR(WEEKDAY(D64)=2,WEEKDAY(D64)=4),2,3),"")</f>
         <v>46325</v>
       </c>
-      <c r="E66" s="27" t="s">
+      <c r="E66" s="28" t="s">
         <v>15</v>
       </c>
       <c r="F66" s="17"/>
-      <c r="G66" s="27"/>
-      <c r="H66" s="28"/>
-      <c r="I66" s="29"/>
-      <c r="J66" s="25"/>
-      <c r="K66" s="26"/>
-    </row>
-    <row r="67" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B67" s="25"/>
-      <c r="C67" s="31"/>
-      <c r="D67" s="28"/>
-      <c r="E67" s="27"/>
+      <c r="G66" s="28"/>
+      <c r="H66" s="29"/>
+      <c r="I66" s="30"/>
+      <c r="J66" s="26"/>
+      <c r="K66" s="27"/>
+    </row>
+    <row r="67" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B67" s="26"/>
+      <c r="C67" s="32"/>
+      <c r="D67" s="29"/>
+      <c r="E67" s="28"/>
       <c r="F67" s="17"/>
-      <c r="G67" s="27"/>
-      <c r="H67" s="28"/>
-      <c r="I67" s="29"/>
-      <c r="J67" s="25"/>
-      <c r="K67" s="26"/>
+      <c r="G67" s="28"/>
+      <c r="H67" s="29"/>
+      <c r="I67" s="30"/>
+      <c r="J67" s="26"/>
+      <c r="K67" s="27"/>
     </row>
     <row r="68" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A68" s="23" t="n">
+      <c r="A68" s="24" t="n">
         <f aca="false">DATE(D3,D4+3,1)</f>
         <v>46327</v>
       </c>
-      <c r="B68" s="25" t="n">
+      <c r="B68" s="26" t="n">
         <v>11</v>
       </c>
       <c r="C68" s="14" t="n">
@@ -2031,15 +2026,15 @@
         <f aca="false">I65+1</f>
         <v>20</v>
       </c>
-      <c r="J68" s="25" t="n">
+      <c r="J68" s="26" t="n">
         <v>11</v>
       </c>
-      <c r="K68" s="26" t="s">
+      <c r="K68" s="27" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="69" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B69" s="25"/>
+    <row r="69" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B69" s="26"/>
       <c r="C69" s="14"/>
       <c r="D69" s="15"/>
       <c r="E69" s="16"/>
@@ -2048,10 +2043,10 @@
       <c r="H69" s="15"/>
       <c r="I69" s="14"/>
       <c r="J69" s="14"/>
-      <c r="K69" s="26"/>
-    </row>
-    <row r="70" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B70" s="25"/>
+      <c r="K69" s="27"/>
+    </row>
+    <row r="70" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B70" s="26"/>
       <c r="C70" s="20" t="n">
         <f aca="false">C68+1</f>
         <v>31</v>
@@ -2066,60 +2061,60 @@
       <c r="H70" s="15"/>
       <c r="I70" s="14"/>
       <c r="J70" s="14"/>
-      <c r="K70" s="26"/>
-    </row>
-    <row r="71" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B71" s="25"/>
+      <c r="K70" s="27"/>
+    </row>
+    <row r="71" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B71" s="26"/>
       <c r="C71" s="20"/>
       <c r="D71" s="21"/>
       <c r="E71" s="22"/>
       <c r="F71" s="22"/>
-      <c r="G71" s="27"/>
-      <c r="H71" s="28" t="n">
+      <c r="G71" s="28"/>
+      <c r="H71" s="29" t="n">
         <f aca="false">H68+IF(WEEKDAY(H68)=3,2,5)</f>
         <v>46331</v>
       </c>
-      <c r="I71" s="29" t="n">
+      <c r="I71" s="30" t="n">
         <f aca="false">I68+1</f>
         <v>21</v>
       </c>
-      <c r="J71" s="25"/>
-      <c r="K71" s="26"/>
+      <c r="J71" s="26"/>
+      <c r="K71" s="27"/>
     </row>
     <row r="72" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B72" s="25"/>
-      <c r="C72" s="31" t="n">
+      <c r="B72" s="26"/>
+      <c r="C72" s="32" t="n">
         <f aca="false">C70+1</f>
         <v>32</v>
       </c>
-      <c r="D72" s="28" t="n">
+      <c r="D72" s="29" t="n">
         <f aca="false">IF(D71="",D70+IF(OR(WEEKDAY(D70)=2,WEEKDAY(D70)=4),2,3),"")</f>
         <v>46332</v>
       </c>
-      <c r="E72" s="27" t="s">
+      <c r="E72" s="28" t="s">
         <v>15</v>
       </c>
       <c r="F72" s="17"/>
-      <c r="G72" s="27"/>
-      <c r="H72" s="28"/>
-      <c r="I72" s="29"/>
-      <c r="J72" s="25"/>
-      <c r="K72" s="26"/>
-    </row>
-    <row r="73" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B73" s="25"/>
-      <c r="C73" s="31"/>
-      <c r="D73" s="28"/>
-      <c r="E73" s="27"/>
+      <c r="G72" s="28"/>
+      <c r="H72" s="29"/>
+      <c r="I72" s="30"/>
+      <c r="J72" s="26"/>
+      <c r="K72" s="27"/>
+    </row>
+    <row r="73" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B73" s="26"/>
+      <c r="C73" s="32"/>
+      <c r="D73" s="29"/>
+      <c r="E73" s="28"/>
       <c r="F73" s="17"/>
-      <c r="G73" s="27"/>
-      <c r="H73" s="28"/>
-      <c r="I73" s="29"/>
-      <c r="J73" s="25"/>
-      <c r="K73" s="26"/>
+      <c r="G73" s="28"/>
+      <c r="H73" s="29"/>
+      <c r="I73" s="30"/>
+      <c r="J73" s="26"/>
+      <c r="K73" s="27"/>
     </row>
     <row r="74" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B74" s="25" t="n">
+      <c r="B74" s="26" t="n">
         <v>12</v>
       </c>
       <c r="C74" s="14" t="n">
@@ -2143,15 +2138,15 @@
         <f aca="false">I71+1</f>
         <v>22</v>
       </c>
-      <c r="J74" s="25" t="n">
+      <c r="J74" s="26" t="n">
         <v>12</v>
       </c>
-      <c r="K74" s="26" t="s">
+      <c r="K74" s="27" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="75" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B75" s="25"/>
+    <row r="75" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B75" s="26"/>
       <c r="C75" s="14"/>
       <c r="D75" s="15"/>
       <c r="E75" s="16"/>
@@ -2160,10 +2155,10 @@
       <c r="H75" s="15"/>
       <c r="I75" s="14"/>
       <c r="J75" s="14"/>
-      <c r="K75" s="26"/>
-    </row>
-    <row r="76" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B76" s="25"/>
+      <c r="K75" s="27"/>
+    </row>
+    <row r="76" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B76" s="26"/>
       <c r="C76" s="20" t="n">
         <f aca="false">C74+1</f>
         <v>34</v>
@@ -2178,60 +2173,60 @@
       <c r="H76" s="15"/>
       <c r="I76" s="14"/>
       <c r="J76" s="14"/>
-      <c r="K76" s="26"/>
-    </row>
-    <row r="77" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B77" s="25"/>
+      <c r="K76" s="27"/>
+    </row>
+    <row r="77" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B77" s="26"/>
       <c r="C77" s="20"/>
       <c r="D77" s="21"/>
       <c r="E77" s="22"/>
       <c r="F77" s="17"/>
-      <c r="G77" s="27"/>
-      <c r="H77" s="28" t="n">
+      <c r="G77" s="28"/>
+      <c r="H77" s="29" t="n">
         <f aca="false">H74+IF(WEEKDAY(H74)=3,2,5)</f>
         <v>46338</v>
       </c>
-      <c r="I77" s="29" t="n">
+      <c r="I77" s="30" t="n">
         <f aca="false">I74+1</f>
         <v>23</v>
       </c>
-      <c r="J77" s="25"/>
-      <c r="K77" s="26"/>
+      <c r="J77" s="26"/>
+      <c r="K77" s="27"/>
     </row>
     <row r="78" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B78" s="25"/>
-      <c r="C78" s="31" t="n">
+      <c r="B78" s="26"/>
+      <c r="C78" s="32" t="n">
         <f aca="false">C76+1</f>
         <v>35</v>
       </c>
-      <c r="D78" s="28" t="n">
+      <c r="D78" s="29" t="n">
         <f aca="false">IF(D77="",D76+IF(OR(WEEKDAY(D76)=2,WEEKDAY(D76)=4),2,3),"")</f>
         <v>46339</v>
       </c>
-      <c r="E78" s="27" t="s">
+      <c r="E78" s="28" t="s">
         <v>15</v>
       </c>
       <c r="F78" s="17"/>
-      <c r="G78" s="27"/>
-      <c r="H78" s="28"/>
-      <c r="I78" s="29"/>
-      <c r="J78" s="25"/>
-      <c r="K78" s="26"/>
-    </row>
-    <row r="79" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B79" s="25"/>
-      <c r="C79" s="31"/>
-      <c r="D79" s="28"/>
-      <c r="E79" s="27"/>
+      <c r="G78" s="28"/>
+      <c r="H78" s="29"/>
+      <c r="I78" s="30"/>
+      <c r="J78" s="26"/>
+      <c r="K78" s="27"/>
+    </row>
+    <row r="79" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B79" s="26"/>
+      <c r="C79" s="32"/>
+      <c r="D79" s="29"/>
+      <c r="E79" s="28"/>
       <c r="F79" s="17"/>
-      <c r="G79" s="27"/>
-      <c r="H79" s="28"/>
-      <c r="I79" s="29"/>
-      <c r="J79" s="25"/>
-      <c r="K79" s="26"/>
+      <c r="G79" s="28"/>
+      <c r="H79" s="29"/>
+      <c r="I79" s="30"/>
+      <c r="J79" s="26"/>
+      <c r="K79" s="27"/>
     </row>
     <row r="80" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B80" s="25" t="n">
+      <c r="B80" s="26" t="n">
         <v>13</v>
       </c>
       <c r="C80" s="14" t="n">
@@ -2255,15 +2250,15 @@
         <f aca="false">I77+1</f>
         <v>24</v>
       </c>
-      <c r="J80" s="25" t="n">
+      <c r="J80" s="26" t="n">
         <v>13</v>
       </c>
-      <c r="K80" s="26" t="s">
+      <c r="K80" s="27" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B81" s="25"/>
+      <c r="B81" s="26"/>
       <c r="C81" s="14"/>
       <c r="D81" s="15"/>
       <c r="E81" s="16"/>
@@ -2272,10 +2267,10 @@
       <c r="H81" s="15"/>
       <c r="I81" s="14"/>
       <c r="J81" s="14"/>
-      <c r="K81" s="26"/>
+      <c r="K81" s="27"/>
     </row>
     <row r="82" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B82" s="25"/>
+      <c r="B82" s="26"/>
       <c r="C82" s="20" t="n">
         <f aca="false">C80+1</f>
         <v>37</v>
@@ -2290,33 +2285,33 @@
       <c r="H82" s="15"/>
       <c r="I82" s="14"/>
       <c r="J82" s="14"/>
-      <c r="K82" s="26"/>
+      <c r="K82" s="27"/>
     </row>
     <row r="83" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B83" s="25"/>
+      <c r="B83" s="26"/>
       <c r="C83" s="20"/>
       <c r="D83" s="21"/>
       <c r="E83" s="33"/>
       <c r="F83" s="17"/>
-      <c r="G83" s="27"/>
-      <c r="H83" s="28" t="n">
+      <c r="G83" s="28"/>
+      <c r="H83" s="29" t="n">
         <f aca="false">H80+IF(WEEKDAY(H80)=3,2,5)</f>
         <v>46345</v>
       </c>
-      <c r="I83" s="29" t="n">
+      <c r="I83" s="30" t="n">
         <f aca="false">I80+1</f>
         <v>25</v>
       </c>
-      <c r="J83" s="25"/>
-      <c r="K83" s="26"/>
+      <c r="J83" s="26"/>
+      <c r="K83" s="27"/>
     </row>
     <row r="84" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B84" s="25"/>
-      <c r="C84" s="31" t="n">
+      <c r="B84" s="26"/>
+      <c r="C84" s="32" t="n">
         <f aca="false">C82+1</f>
         <v>38</v>
       </c>
-      <c r="D84" s="28" t="n">
+      <c r="D84" s="29" t="n">
         <f aca="false">IF(D83="",D82+IF(OR(WEEKDAY(D82)=2,WEEKDAY(D82)=4),2,3),"")</f>
         <v>46346</v>
       </c>
@@ -2324,26 +2319,26 @@
         <v>15</v>
       </c>
       <c r="F84" s="17"/>
-      <c r="G84" s="27"/>
-      <c r="H84" s="28"/>
-      <c r="I84" s="29"/>
-      <c r="J84" s="25"/>
-      <c r="K84" s="26"/>
+      <c r="G84" s="28"/>
+      <c r="H84" s="29"/>
+      <c r="I84" s="30"/>
+      <c r="J84" s="26"/>
+      <c r="K84" s="27"/>
     </row>
     <row r="85" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B85" s="25"/>
-      <c r="C85" s="31"/>
-      <c r="D85" s="28"/>
+      <c r="B85" s="26"/>
+      <c r="C85" s="32"/>
+      <c r="D85" s="29"/>
       <c r="E85" s="34"/>
       <c r="F85" s="17"/>
-      <c r="G85" s="27"/>
-      <c r="H85" s="28"/>
-      <c r="I85" s="29"/>
-      <c r="J85" s="25"/>
-      <c r="K85" s="26"/>
+      <c r="G85" s="28"/>
+      <c r="H85" s="29"/>
+      <c r="I85" s="30"/>
+      <c r="J85" s="26"/>
+      <c r="K85" s="27"/>
     </row>
     <row r="86" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B86" s="25" t="n">
+      <c r="B86" s="26" t="n">
         <v>14</v>
       </c>
       <c r="C86" s="14" t="n">
@@ -2367,13 +2362,13 @@
         <f aca="false">I83+1</f>
         <v>26</v>
       </c>
-      <c r="J86" s="25" t="n">
+      <c r="J86" s="26" t="n">
         <v>14</v>
       </c>
-      <c r="K86" s="26"/>
-    </row>
-    <row r="87" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B87" s="25"/>
+      <c r="K86" s="27"/>
+    </row>
+    <row r="87" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B87" s="26"/>
       <c r="C87" s="14"/>
       <c r="D87" s="15"/>
       <c r="E87" s="16"/>
@@ -2382,10 +2377,10 @@
       <c r="H87" s="15"/>
       <c r="I87" s="14"/>
       <c r="J87" s="14"/>
-      <c r="K87" s="26"/>
+      <c r="K87" s="27"/>
     </row>
     <row r="88" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B88" s="25"/>
+      <c r="B88" s="26"/>
       <c r="C88" s="20"/>
       <c r="D88" s="21" t="n">
         <f aca="false">IF(D87="",D86+IF(OR(WEEKDAY(D86)=2,WEEKDAY(D86)=4),2,3),"")</f>
@@ -2399,10 +2394,10 @@
       <c r="H88" s="15"/>
       <c r="I88" s="14"/>
       <c r="J88" s="14"/>
-      <c r="K88" s="26"/>
+      <c r="K88" s="27"/>
     </row>
     <row r="89" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B89" s="25"/>
+      <c r="B89" s="26"/>
       <c r="C89" s="20"/>
       <c r="D89" s="21"/>
       <c r="E89" s="35"/>
@@ -2410,18 +2405,18 @@
       <c r="G89" s="36" t="s">
         <v>45</v>
       </c>
-      <c r="H89" s="28" t="n">
+      <c r="H89" s="29" t="n">
         <f aca="false">H86+IF(WEEKDAY(H86)=3,2,5)</f>
         <v>46352</v>
       </c>
-      <c r="I89" s="29"/>
-      <c r="J89" s="25"/>
-      <c r="K89" s="26"/>
+      <c r="I89" s="30"/>
+      <c r="J89" s="26"/>
+      <c r="K89" s="27"/>
     </row>
     <row r="90" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B90" s="25"/>
-      <c r="C90" s="31"/>
-      <c r="D90" s="28" t="n">
+      <c r="B90" s="26"/>
+      <c r="C90" s="32"/>
+      <c r="D90" s="29" t="n">
         <f aca="false">IF(D89="",D88+IF(OR(WEEKDAY(D88)=2,WEEKDAY(D88)=4),2,3),"")</f>
         <v>46353</v>
       </c>
@@ -2430,25 +2425,25 @@
       </c>
       <c r="F90" s="17"/>
       <c r="G90" s="36"/>
-      <c r="H90" s="28"/>
-      <c r="I90" s="29"/>
-      <c r="J90" s="25"/>
-      <c r="K90" s="26"/>
-    </row>
-    <row r="91" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B91" s="25"/>
-      <c r="C91" s="31"/>
-      <c r="D91" s="28"/>
+      <c r="H90" s="29"/>
+      <c r="I90" s="30"/>
+      <c r="J90" s="26"/>
+      <c r="K90" s="27"/>
+    </row>
+    <row r="91" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B91" s="26"/>
+      <c r="C91" s="32"/>
+      <c r="D91" s="29"/>
       <c r="E91" s="36"/>
       <c r="F91" s="17"/>
       <c r="G91" s="36"/>
-      <c r="H91" s="28"/>
-      <c r="I91" s="29"/>
-      <c r="J91" s="25"/>
-      <c r="K91" s="26"/>
+      <c r="H91" s="29"/>
+      <c r="I91" s="30"/>
+      <c r="J91" s="26"/>
+      <c r="K91" s="27"/>
     </row>
     <row r="92" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A92" s="0"/>
+      <c r="A92" s="23"/>
       <c r="B92" s="14" t="n">
         <v>15</v>
       </c>
@@ -2480,8 +2475,8 @@
         <v>47</v>
       </c>
     </row>
-    <row r="93" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A93" s="23" t="n">
+    <row r="93" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A93" s="24" t="n">
         <f aca="false">DATE(D3,D4+4,1)</f>
         <v>46357</v>
       </c>
@@ -2496,8 +2491,8 @@
       <c r="J93" s="14"/>
       <c r="K93" s="18"/>
     </row>
-    <row r="94" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A94" s="0"/>
+    <row r="94" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A94" s="23"/>
       <c r="B94" s="14"/>
       <c r="C94" s="20" t="n">
         <f aca="false">C92+1</f>
@@ -2552,7 +2547,7 @@
       <c r="J96" s="14"/>
       <c r="K96" s="18"/>
     </row>
-    <row r="97" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="97" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B97" s="14"/>
       <c r="C97" s="20"/>
       <c r="D97" s="21"/>
@@ -2632,7 +2627,7 @@
       <c r="J101" s="14"/>
       <c r="K101" s="18"/>
     </row>
-    <row r="102" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="102" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B102" s="14"/>
       <c r="C102" s="20"/>
       <c r="D102" s="21" t="n">
@@ -2647,7 +2642,7 @@
       <c r="J102" s="14"/>
       <c r="K102" s="18"/>
     </row>
-    <row r="103" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="103" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B103" s="14"/>
       <c r="C103" s="14"/>
       <c r="D103" s="21"/>
@@ -2974,7 +2969,7 @@
       <formula>"not(isblank(address(row(),c)))"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B98 E98:F98 B102 E102:F102">
+  <conditionalFormatting sqref="B98 E98:G98 B102 E102:G102">
     <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
       <formula>"not(isblank(address(row(),c)))"</formula>
     </cfRule>
@@ -2989,16 +2984,6 @@
       <formula>"not(isblank(address(row(),c)))"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G98">
-    <cfRule type="expression" priority="6" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
-      <formula>"not(isblank(address(row(),c)))"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G102">
-    <cfRule type="expression" priority="7" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
-      <formula>"not(isblank(address(row(),c)))"</formula>
-    </cfRule>
-  </conditionalFormatting>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>